<commit_message>
Added currency to the Sales Data Row
</commit_message>
<xml_diff>
--- a/Combining Multiple Excel Files & Sheets Automatically (Power Query)/Cleaned Sales Data.xlsx
+++ b/Combining Multiple Excel Files & Sheets Automatically (Power Query)/Cleaned Sales Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\louis\Downloads\repo\power-query-data-cleaning-automation\Combining Multiple Excel Files &amp; Sheets Automatically (Power Query)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{184BAB24-1973-4672-97AD-8195F5DD9F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{573E3FA2-826A-43C7-A54F-725C6CD7D5C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7526E2B5-70C3-47BE-9CEF-E95001061655}"/>
   </bookViews>
@@ -303,7 +303,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -329,15 +339,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
@@ -382,7 +395,7 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{6AAE2018-B5E4-443F-A559-F4C437927B0A}" uniqueName="1" name="Category" queryTableFieldId="1" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{4B32FEB7-5D3B-4A90-844D-DE8C78C929E7}" uniqueName="2" name="Product" queryTableFieldId="2" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{3C6FB85F-636D-46D3-BABC-3C102841E5CF}" uniqueName="3" name="Sales" queryTableFieldId="3"/>
+    <tableColumn id="3" xr3:uid="{3C6FB85F-636D-46D3-BABC-3C102841E5CF}" uniqueName="3" name="Sales" queryTableFieldId="3" dataCellStyle="Currency"/>
     <tableColumn id="4" xr3:uid="{D2324871-ED1E-4907-9E11-5DAEC13E0F93}" uniqueName="4" name="Date" queryTableFieldId="4" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -691,7 +704,7 @@
   <cols>
     <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -702,7 +715,7 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
@@ -716,7 +729,7 @@
       <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="3">
         <v>986.88240000000008</v>
       </c>
       <c r="D2" s="2">
@@ -730,7 +743,7 @@
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="3">
         <v>256.15800000000002</v>
       </c>
       <c r="D3" s="2">
@@ -744,7 +757,7 @@
       <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="3">
         <v>400.608</v>
       </c>
       <c r="D4" s="2">
@@ -758,7 +771,7 @@
       <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="3">
         <v>15346.828100000001</v>
       </c>
       <c r="D5" s="2">
@@ -772,7 +785,7 @@
       <c r="B6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="3">
         <v>455.25290000000001</v>
       </c>
       <c r="D6" s="2">
@@ -786,7 +799,7 @@
       <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="3">
         <v>4715.0298999999995</v>
       </c>
       <c r="D7" s="2">
@@ -800,7 +813,7 @@
       <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="3">
         <v>2126.0579000000002</v>
       </c>
       <c r="D8" s="2">
@@ -814,7 +827,7 @@
       <c r="B9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="3">
         <v>543.1748</v>
       </c>
       <c r="D9" s="2">
@@ -828,7 +841,7 @@
       <c r="B10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="3">
         <v>431.42399999999998</v>
       </c>
       <c r="D10" s="2">
@@ -842,7 +855,7 @@
       <c r="B11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="3">
         <v>1695.2758999999999</v>
       </c>
       <c r="D11" s="2">
@@ -856,7 +869,7 @@
       <c r="B12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="3">
         <v>932.4194</v>
       </c>
       <c r="D12" s="2">
@@ -870,7 +883,7 @@
       <c r="B13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="3">
         <v>905.99040000000002</v>
       </c>
       <c r="D13" s="2">
@@ -884,7 +897,7 @@
       <c r="B14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="3">
         <v>770.4</v>
       </c>
       <c r="D14" s="2">
@@ -898,7 +911,7 @@
       <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="3">
         <v>3050.7839999999997</v>
       </c>
       <c r="D15" s="2">
@@ -912,7 +925,7 @@
       <c r="B16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="3">
         <v>158.8201</v>
       </c>
       <c r="D16" s="2">
@@ -926,7 +939,7 @@
       <c r="B17" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="3">
         <v>1951.4232</v>
       </c>
       <c r="D17" s="2">
@@ -940,7 +953,7 @@
       <c r="B18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="3">
         <v>2393.3760000000002</v>
       </c>
       <c r="D18" s="2">
@@ -954,7 +967,7 @@
       <c r="B19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="3">
         <v>1362.0672</v>
       </c>
       <c r="D19" s="2">
@@ -968,7 +981,7 @@
       <c r="B20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="3">
         <v>1335.3600000000001</v>
       </c>
       <c r="D20" s="2">
@@ -982,7 +995,7 @@
       <c r="B21" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="3">
         <v>1000.7496</v>
       </c>
       <c r="D21" s="2">
@@ -996,7 +1009,7 @@
       <c r="B22" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="3">
         <v>1831.5297</v>
       </c>
       <c r="D22" s="2">
@@ -1010,7 +1023,7 @@
       <c r="B23" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="3">
         <v>270.56020000000001</v>
       </c>
       <c r="D23" s="2">
@@ -1024,7 +1037,7 @@
       <c r="B24" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="3">
         <v>2722.7647999999999</v>
       </c>
       <c r="D24" s="2">
@@ -1038,7 +1051,7 @@
       <c r="B25" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="3">
         <v>2477.3175000000001</v>
       </c>
       <c r="D25" s="2">
@@ -1052,7 +1065,7 @@
       <c r="B26" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="3">
         <v>272.20800000000003</v>
       </c>
       <c r="D26" s="2">
@@ -1066,7 +1079,7 @@
       <c r="B27" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="3">
         <v>441.6746</v>
       </c>
       <c r="D27" s="2">
@@ -1080,7 +1093,7 @@
       <c r="B28" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="3">
         <v>593.34709999999995</v>
       </c>
       <c r="D28" s="2">
@@ -1094,7 +1107,7 @@
       <c r="B29" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="3">
         <v>3002.3344000000002</v>
       </c>
       <c r="D29" s="2">
@@ -1108,7 +1121,7 @@
       <c r="B30" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="3">
         <v>1489.0333999999998</v>
       </c>
       <c r="D30" s="2">
@@ -1122,7 +1135,7 @@
       <c r="B31" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="3">
         <v>163.58160000000001</v>
       </c>
       <c r="D31" s="2">
@@ -1136,7 +1149,7 @@
       <c r="B32" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="3">
         <v>146.10850000000002</v>
       </c>
       <c r="D32" s="2">
@@ -1150,7 +1163,7 @@
       <c r="B33" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="3">
         <v>1309.9154000000001</v>
       </c>
       <c r="D33" s="2">
@@ -1164,7 +1177,7 @@
       <c r="B34" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="3">
         <v>603.69400000000007</v>
       </c>
       <c r="D34" s="2">
@@ -1178,7 +1191,7 @@
       <c r="B35" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C35">
+      <c r="C35" s="3">
         <v>907.25299999999993</v>
       </c>
       <c r="D35" s="2">
@@ -1192,7 +1205,7 @@
       <c r="B36" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="3">
         <v>2576.4850999999999</v>
       </c>
       <c r="D36" s="2">
@@ -1206,7 +1219,7 @@
       <c r="B37" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="3">
         <v>6764.1120000000001</v>
       </c>
       <c r="D37" s="2">
@@ -1220,7 +1233,7 @@
       <c r="B38" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="3">
         <v>1034.5616</v>
       </c>
       <c r="D38" s="2">
@@ -1234,7 +1247,7 @@
       <c r="B39" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="3">
         <v>3822.1469999999999</v>
       </c>
       <c r="D39" s="2">
@@ -1248,7 +1261,7 @@
       <c r="B40" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="3">
         <v>792.74159999999995</v>
       </c>
       <c r="D40" s="2">
@@ -1262,7 +1275,7 @@
       <c r="B41" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="3">
         <v>5839.5249999999996</v>
       </c>
       <c r="D41" s="2">
@@ -1276,7 +1289,7 @@
       <c r="B42" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="3">
         <v>4183.8069999999998</v>
       </c>
       <c r="D42" s="2">
@@ -1290,7 +1303,7 @@
       <c r="B43" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="3">
         <v>195.6602</v>
       </c>
       <c r="D43" s="2">
@@ -1304,7 +1317,7 @@
       <c r="B44" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="3">
         <v>272.45409999999998</v>
       </c>
       <c r="D44" s="2">
@@ -1318,7 +1331,7 @@
       <c r="B45" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="3">
         <v>3074.538</v>
       </c>
       <c r="D45" s="2">
@@ -1332,7 +1345,7 @@
       <c r="B46" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="3">
         <v>1627.0848000000001</v>
       </c>
       <c r="D46" s="2">
@@ -1346,7 +1359,7 @@
       <c r="B47" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="3">
         <v>2162.3951000000002</v>
       </c>
       <c r="D47" s="2">
@@ -1360,7 +1373,7 @@
       <c r="B48" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="3">
         <v>5042.4926999999998</v>
       </c>
       <c r="D48" s="2">
@@ -1374,7 +1387,7 @@
       <c r="B49" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="3">
         <v>3889.5569999999998</v>
       </c>
       <c r="D49" s="2">
@@ -1388,7 +1401,7 @@
       <c r="B50" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="3">
         <v>833.63700000000006</v>
       </c>
       <c r="D50" s="2">
@@ -1402,7 +1415,7 @@
       <c r="B51" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="3">
         <v>11087.372100000001</v>
       </c>
       <c r="D51" s="2">
@@ -1416,7 +1429,7 @@
       <c r="B52" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="3">
         <v>603.99360000000001</v>
       </c>
       <c r="D52" s="2">
@@ -1430,7 +1443,7 @@
       <c r="B53" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C53">
+      <c r="C53" s="3">
         <v>78.869699999999995</v>
       </c>
       <c r="D53" s="2">
@@ -1444,7 +1457,7 @@
       <c r="B54" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="3">
         <v>1093.9038</v>
       </c>
       <c r="D54" s="2">
@@ -1458,7 +1471,7 @@
       <c r="B55" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C55">
+      <c r="C55" s="3">
         <v>758.03080000000011</v>
       </c>
       <c r="D55" s="2">
@@ -1472,7 +1485,7 @@
       <c r="B56" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C56">
+      <c r="C56" s="3">
         <v>1820.0058000000001</v>
       </c>
       <c r="D56" s="2">
@@ -1486,7 +1499,7 @@
       <c r="B57" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C57">
+      <c r="C57" s="3">
         <v>4122.2605999999996</v>
       </c>
       <c r="D57" s="2">
@@ -1500,7 +1513,7 @@
       <c r="B58" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C58">
+      <c r="C58" s="3">
         <v>1383.3173999999999</v>
       </c>
       <c r="D58" s="2">
@@ -1514,7 +1527,7 @@
       <c r="B59" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C59">
+      <c r="C59" s="3">
         <v>1478.9754</v>
       </c>
       <c r="D59" s="2">
@@ -1528,7 +1541,7 @@
       <c r="B60" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C60">
+      <c r="C60" s="3">
         <v>2695.3728000000001</v>
       </c>
       <c r="D60" s="2">
@@ -1542,7 +1555,7 @@
       <c r="B61" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C61">
+      <c r="C61" s="3">
         <v>4005.4486999999999</v>
       </c>
       <c r="D61" s="2">
@@ -1556,7 +1569,7 @@
       <c r="B62" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C62">
+      <c r="C62" s="3">
         <v>514.03870000000006</v>
       </c>
       <c r="D62" s="2">
@@ -1570,7 +1583,7 @@
       <c r="B63" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C63">
+      <c r="C63" s="3">
         <v>2554.0387000000001</v>
       </c>
       <c r="D63" s="2">
@@ -1584,7 +1597,7 @@
       <c r="B64" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C64">
+      <c r="C64" s="3">
         <v>1514.0387000000001</v>
       </c>
       <c r="D64" s="2">
@@ -1598,7 +1611,7 @@
       <c r="B65" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C65">
+      <c r="C65" s="3">
         <v>115.04639999999999</v>
       </c>
       <c r="D65" s="2">
@@ -1612,7 +1625,7 @@
       <c r="B66" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C66">
+      <c r="C66" s="3">
         <v>8792.0936999999994</v>
       </c>
       <c r="D66" s="2">
@@ -1626,7 +1639,7 @@
       <c r="B67" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C67">
+      <c r="C67" s="3">
         <v>3719.4163000000003</v>
       </c>
       <c r="D67" s="2">
@@ -1640,7 +1653,7 @@
       <c r="B68" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C68">
+      <c r="C68" s="3">
         <v>2244.9456</v>
       </c>
       <c r="D68" s="2">
@@ -1654,7 +1667,7 @@
       <c r="B69" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C69">
+      <c r="C69" s="3">
         <v>2022.3</v>
       </c>
       <c r="D69" s="2">
@@ -1668,7 +1681,7 @@
       <c r="B70" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C70">
+      <c r="C70" s="3">
         <v>1022.3</v>
       </c>
       <c r="D70" s="2">
@@ -1682,7 +1695,7 @@
       <c r="B71" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C71">
+      <c r="C71" s="3">
         <v>1222.3</v>
       </c>
       <c r="D71" s="2">
@@ -1696,7 +1709,7 @@
       <c r="B72" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C72">
+      <c r="C72" s="3">
         <v>522.29999999999995</v>
       </c>
       <c r="D72" s="2">
@@ -1710,7 +1723,7 @@
       <c r="B73" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C73">
+      <c r="C73" s="3">
         <v>1228.9967999999999</v>
       </c>
       <c r="D73" s="2">
@@ -1724,7 +1737,7 @@
       <c r="B74" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C74">
+      <c r="C74" s="3">
         <v>2202.0942999999997</v>
       </c>
       <c r="D74" s="2">
@@ -1738,7 +1751,7 @@
       <c r="B75" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C75">
+      <c r="C75" s="3">
         <v>1247.7556999999999</v>
       </c>
       <c r="D75" s="2">
@@ -1752,7 +1765,7 @@
       <c r="B76" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C76">
+      <c r="C76" s="3">
         <v>6694.9762000000001</v>
       </c>
       <c r="D76" s="2">
@@ -1766,7 +1779,7 @@
       <c r="B77" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C77">
+      <c r="C77" s="3">
         <v>200.85430000000002</v>
       </c>
       <c r="D77" s="2">
@@ -1780,7 +1793,7 @@
       <c r="B78" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C78">
+      <c r="C78" s="3">
         <v>1355.7855999999999</v>
       </c>
       <c r="D78" s="2">
@@ -1794,7 +1807,7 @@
       <c r="B79" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C79">
+      <c r="C79" s="3">
         <v>3235.1853999999998</v>
       </c>
       <c r="D79" s="2">
@@ -1808,7 +1821,7 @@
       <c r="B80" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C80">
+      <c r="C80" s="3">
         <v>457.8</v>
       </c>
       <c r="D80" s="2">
@@ -1822,7 +1835,7 @@
       <c r="B81" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C81">
+      <c r="C81" s="3">
         <v>1337.9204999999999</v>
       </c>
       <c r="D81" s="2">
@@ -1836,7 +1849,7 @@
       <c r="B82" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C82">
+      <c r="C82" s="3">
         <v>1129.6651000000002</v>
       </c>
       <c r="D82" s="2">
@@ -1850,7 +1863,7 @@
       <c r="B83" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C83">
+      <c r="C83" s="3">
         <v>1540.9548</v>
       </c>
       <c r="D83" s="2">
@@ -1864,7 +1877,7 @@
       <c r="B84" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C84">
+      <c r="C84" s="3">
         <v>158.70400000000001</v>
       </c>
       <c r="D84" s="2">
@@ -1878,7 +1891,7 @@
       <c r="B85" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C85">
+      <c r="C85" s="3">
         <v>1224.7021999999999</v>
       </c>
       <c r="D85" s="2">
@@ -1892,7 +1905,7 @@
       <c r="B86" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C86">
+      <c r="C86" s="3">
         <v>307.88139999999999</v>
       </c>
       <c r="D86" s="2">
@@ -1906,7 +1919,7 @@
       <c r="B87" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C87">
+      <c r="C87" s="3">
         <v>1471.5436</v>
       </c>
       <c r="D87" s="2">
@@ -1920,7 +1933,7 @@
       <c r="B88" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C88">
+      <c r="C88" s="3">
         <v>2136.4</v>
       </c>
       <c r="D88" s="2">
@@ -1934,7 +1947,7 @@
       <c r="B89" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C89">
+      <c r="C89" s="3">
         <v>1251.0365999999999</v>
       </c>
       <c r="D89" s="2">
@@ -1948,7 +1961,7 @@
       <c r="B90" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C90">
+      <c r="C90" s="3">
         <v>2411.7339999999999</v>
       </c>
       <c r="D90" s="2">
@@ -1962,7 +1975,7 @@
       <c r="B91" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C91">
+      <c r="C91" s="3">
         <v>2065.1358</v>
       </c>
       <c r="D91" s="2">
@@ -1976,7 +1989,7 @@
       <c r="B92" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C92">
+      <c r="C92" s="3">
         <v>3161.1743999999999</v>
       </c>
       <c r="D92" s="2">
@@ -1990,7 +2003,7 @@
       <c r="B93" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C93">
+      <c r="C93" s="3">
         <v>771.74180000000001</v>
       </c>
       <c r="D93" s="2">
@@ -2004,7 +2017,7 @@
       <c r="B94" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C94">
+      <c r="C94" s="3">
         <v>78.79610000000001</v>
       </c>
       <c r="D94" s="2">
@@ -2018,7 +2031,7 @@
       <c r="B95" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C95">
+      <c r="C95" s="3">
         <v>2044.4694000000002</v>
       </c>
       <c r="D95" s="2">
@@ -2032,7 +2045,7 @@
       <c r="B96" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C96">
+      <c r="C96" s="3">
         <v>955.65750000000003</v>
       </c>
       <c r="D96" s="2">
@@ -2046,7 +2059,7 @@
       <c r="B97" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C97">
+      <c r="C97" s="3">
         <v>2116.9871000000003</v>
       </c>
       <c r="D97" s="2">
@@ -2060,7 +2073,7 @@
       <c r="B98" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C98">
+      <c r="C98" s="3">
         <v>2344.6990000000001</v>
       </c>
       <c r="D98" s="2">
@@ -2074,7 +2087,7 @@
       <c r="B99" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C99">
+      <c r="C99" s="3">
         <v>526.08849999999995</v>
       </c>
       <c r="D99" s="2">
@@ -2088,7 +2101,7 @@
       <c r="B100" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C100">
+      <c r="C100" s="3">
         <v>1423.9432999999999</v>
       </c>
       <c r="D100" s="2">
@@ -2102,7 +2115,7 @@
       <c r="B101" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C101">
+      <c r="C101" s="3">
         <v>1983.4185</v>
       </c>
       <c r="D101" s="2">
@@ -2116,7 +2129,7 @@
       <c r="B102" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C102">
+      <c r="C102" s="3">
         <v>2264.5839999999998</v>
       </c>
       <c r="D102" s="2">
@@ -2130,7 +2143,7 @@
       <c r="B103" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C103">
+      <c r="C103" s="3">
         <v>2009.2842000000001</v>
       </c>
       <c r="D103" s="2">
@@ -2144,7 +2157,7 @@
       <c r="B104" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C104">
+      <c r="C104" s="3">
         <v>1994.2967000000001</v>
       </c>
       <c r="D104" s="2">
@@ -2158,7 +2171,7 @@
       <c r="B105" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C105">
+      <c r="C105" s="3">
         <v>3531.6</v>
       </c>
       <c r="D105" s="2">
@@ -2172,7 +2185,7 @@
       <c r="B106" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C106">
+      <c r="C106" s="3">
         <v>1309.9154000000001</v>
       </c>
       <c r="D106" s="2">
@@ -2186,7 +2199,7 @@
       <c r="B107" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C107">
+      <c r="C107" s="3">
         <v>603.69400000000007</v>
       </c>
       <c r="D107" s="2">
@@ -2200,7 +2213,7 @@
       <c r="B108" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C108">
+      <c r="C108" s="3">
         <v>907.25299999999993</v>
       </c>
       <c r="D108" s="2">
@@ -2214,7 +2227,7 @@
       <c r="B109" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C109">
+      <c r="C109" s="3">
         <v>807.25300000000004</v>
       </c>
       <c r="D109" s="2">
@@ -2228,7 +2241,7 @@
       <c r="B110" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C110">
+      <c r="C110" s="3">
         <v>3107.2530000000002</v>
       </c>
       <c r="D110" s="2">
@@ -2242,7 +2255,7 @@
       <c r="B111" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C111">
+      <c r="C111" s="3">
         <v>10189.8868</v>
       </c>
       <c r="D111" s="2">
@@ -2256,7 +2269,7 @@
       <c r="B112" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C112">
+      <c r="C112" s="3">
         <v>2880.8045999999999</v>
       </c>
       <c r="D112" s="2">
@@ -2270,7 +2283,7 @@
       <c r="B113" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C113">
+      <c r="C113" s="3">
         <v>112.7932</v>
       </c>
       <c r="D113" s="2">
@@ -2284,7 +2297,7 @@
       <c r="B114" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C114">
+      <c r="C114" s="3">
         <v>1446.9313999999999</v>
       </c>
       <c r="D114" s="2">
@@ -2298,7 +2311,7 @@
       <c r="B115" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C115">
+      <c r="C115" s="3">
         <v>4778.0586000000003</v>
       </c>
       <c r="D115" s="2">
@@ -2312,7 +2325,7 @@
       <c r="B116" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C116">
+      <c r="C116" s="3">
         <v>3432.0829999999996</v>
       </c>
       <c r="D116" s="2">
@@ -2326,7 +2339,7 @@
       <c r="B117" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C117">
+      <c r="C117" s="3">
         <v>461.4624</v>
       </c>
       <c r="D117" s="2">
@@ -2340,7 +2353,7 @@
       <c r="B118" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C118">
+      <c r="C118" s="3">
         <v>1153.3835000000001</v>
       </c>
       <c r="D118" s="2">
@@ -2354,7 +2367,7 @@
       <c r="B119" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C119">
+      <c r="C119" s="3">
         <v>224.96509999999998</v>
       </c>
       <c r="D119" s="2">
@@ -2368,7 +2381,7 @@
       <c r="B120" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C120">
+      <c r="C120" s="3">
         <v>7085.8065999999999</v>
       </c>
       <c r="D120" s="2">
@@ -2382,7 +2395,7 @@
       <c r="B121" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C121">
+      <c r="C121" s="3">
         <v>3037.9607999999998</v>
       </c>
       <c r="D121" s="2">
@@ -2396,7 +2409,7 @@
       <c r="B122" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C122">
+      <c r="C122" s="3">
         <v>624.89699999999993</v>
       </c>
       <c r="D122" s="2">
@@ -2410,7 +2423,7 @@
       <c r="B123" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C123">
+      <c r="C123" s="3">
         <v>2640.5904</v>
       </c>
       <c r="D123" s="2">
@@ -2424,7 +2437,7 @@
       <c r="B124" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C124">
+      <c r="C124" s="3">
         <v>387.29879999999997</v>
       </c>
       <c r="D124" s="2">
@@ -2438,7 +2451,7 @@
       <c r="B125" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C125">
+      <c r="C125" s="3">
         <v>1903.4451999999999</v>
       </c>
       <c r="D125" s="2">
@@ -2452,7 +2465,7 @@
       <c r="B126" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C126">
+      <c r="C126" s="3">
         <v>4761.12</v>
       </c>
       <c r="D126" s="2">
@@ -2466,7 +2479,7 @@
       <c r="B127" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C127">
+      <c r="C127" s="3">
         <v>979.43039999999996</v>
       </c>
       <c r="D127" s="2">
@@ -2480,7 +2493,7 @@
       <c r="B128" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C128">
+      <c r="C128" s="3">
         <v>1602.9431</v>
       </c>
       <c r="D128" s="2">
@@ -2494,7 +2507,7 @@
       <c r="B129" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C129">
+      <c r="C129" s="3">
         <v>8160.6337999999996</v>
       </c>
       <c r="D129" s="2">
@@ -2508,7 +2521,7 @@
       <c r="B130" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C130">
+      <c r="C130" s="3">
         <v>660.63810000000001</v>
       </c>
       <c r="D130" s="2">
@@ -2522,7 +2535,7 @@
       <c r="B131" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C131">
+      <c r="C131" s="3">
         <v>1960.6380999999999</v>
       </c>
       <c r="D131" s="2">
@@ -2536,7 +2549,7 @@
       <c r="B132" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C132">
+      <c r="C132" s="3">
         <v>260.63810000000001</v>
       </c>
       <c r="D132" s="2">
@@ -2550,7 +2563,7 @@
       <c r="B133" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C133">
+      <c r="C133" s="3">
         <v>4153.0743999999995</v>
       </c>
       <c r="D133" s="2">
@@ -2564,7 +2577,7 @@
       <c r="B134" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C134">
+      <c r="C134" s="3">
         <v>9286.7999999999993</v>
       </c>
       <c r="D134" s="2">
@@ -2578,7 +2591,7 @@
       <c r="B135" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C135">
+      <c r="C135" s="3">
         <v>1701.6753000000001</v>
       </c>
       <c r="D135" s="2">
@@ -2592,7 +2605,7 @@
       <c r="B136" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C136">
+      <c r="C136" s="3">
         <v>4248.6238000000003</v>
       </c>
       <c r="D136" s="2">
@@ -2606,7 +2619,7 @@
       <c r="B137" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C137">
+      <c r="C137" s="3">
         <v>2517.0389</v>
       </c>
       <c r="D137" s="2">
@@ -2620,7 +2633,7 @@
       <c r="B138" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C138">
+      <c r="C138" s="3">
         <v>531.10249999999996</v>
       </c>
       <c r="D138" s="2">
@@ -2634,7 +2647,7 @@
       <c r="B139" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C139">
+      <c r="C139" s="3">
         <v>429.87419999999997</v>
       </c>
       <c r="D139" s="2">
@@ -2648,7 +2661,7 @@
       <c r="B140" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C140">
+      <c r="C140" s="3">
         <v>2860.7039999999997</v>
       </c>
       <c r="D140" s="2">
@@ -2662,7 +2675,7 @@
       <c r="B141" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C141">
+      <c r="C141" s="3">
         <v>1908.1776</v>
       </c>
       <c r="D141" s="2">
@@ -2676,7 +2689,7 @@
       <c r="B142" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C142">
+      <c r="C142" s="3">
         <v>3041.4160000000002</v>
       </c>
       <c r="D142" s="2">
@@ -2690,7 +2703,7 @@
       <c r="B143" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C143">
+      <c r="C143" s="3">
         <v>1770.72</v>
       </c>
       <c r="D143" s="2">
@@ -2704,7 +2717,7 @@
       <c r="B144" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C144">
+      <c r="C144" s="3">
         <v>396.90559999999999</v>
       </c>
       <c r="D144" s="2">
@@ -2718,7 +2731,7 @@
       <c r="B145" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C145">
+      <c r="C145" s="3">
         <v>4055.3968</v>
       </c>
       <c r="D145" s="2">
@@ -2732,7 +2745,7 @@
       <c r="B146" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C146">
+      <c r="C146" s="3">
         <v>1871.9568000000002</v>
       </c>
       <c r="D146" s="2">
@@ -2746,7 +2759,7 @@
       <c r="B147" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C147">
+      <c r="C147" s="3">
         <v>39.513600000000004</v>
       </c>
       <c r="D147" s="2">
@@ -2760,7 +2773,7 @@
       <c r="B148" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C148">
+      <c r="C148" s="3">
         <v>3606.6239999999998</v>
       </c>
       <c r="D148" s="2">
@@ -2774,7 +2787,7 @@
       <c r="B149" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C149">
+      <c r="C149" s="3">
         <v>1547.6831999999999</v>
       </c>
       <c r="D149" s="2">
@@ -2788,7 +2801,7 @@
       <c r="B150" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C150">
+      <c r="C150" s="3">
         <v>941.30400000000009</v>
       </c>
       <c r="D150" s="2">
@@ -2802,7 +2815,7 @@
       <c r="B151" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C151">
+      <c r="C151" s="3">
         <v>1426.32</v>
       </c>
       <c r="D151" s="2">
@@ -2816,7 +2829,7 @@
       <c r="B152" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C152">
+      <c r="C152" s="3">
         <v>512.51200000000006</v>
       </c>
       <c r="D152" s="2">
@@ -2830,7 +2843,7 @@
       <c r="B153" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C153">
+      <c r="C153" s="3">
         <v>794.39359999999999</v>
       </c>
       <c r="D153" s="2">
@@ -2844,7 +2857,7 @@
       <c r="B154" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C154">
+      <c r="C154" s="3">
         <v>80.348799999999997</v>
       </c>
       <c r="D154" s="2">
@@ -2858,7 +2871,7 @@
       <c r="B155" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C155">
+      <c r="C155" s="3">
         <v>806.4</v>
       </c>
       <c r="D155" s="2">
@@ -2872,7 +2885,7 @@
       <c r="B156" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C156">
+      <c r="C156" s="3">
         <v>2001.3951999999999</v>
       </c>
       <c r="D156" s="2">
@@ -2886,7 +2899,7 @@
       <c r="B157" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C157">
+      <c r="C157" s="3">
         <v>4493.1152000000002</v>
       </c>
       <c r="D157" s="2">
@@ -2900,7 +2913,7 @@
       <c r="B158" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C158">
+      <c r="C158" s="3">
         <v>863.65440000000001</v>
       </c>
       <c r="D158" s="2">
@@ -2914,7 +2927,7 @@
       <c r="B159" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C159">
+      <c r="C159" s="3">
         <v>3480.96</v>
       </c>
       <c r="D159" s="2">
@@ -2928,7 +2941,7 @@
       <c r="B160" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C160">
+      <c r="C160" s="3">
         <v>686.64960000000008</v>
       </c>
       <c r="D160" s="2">
@@ -2942,7 +2955,7 @@
       <c r="B161" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C161">
+      <c r="C161" s="3">
         <v>1624.0895999999998</v>
       </c>
       <c r="D161" s="2">
@@ -2956,7 +2969,7 @@
       <c r="B162" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C162">
+      <c r="C162" s="3">
         <v>311.87519999999995</v>
       </c>
       <c r="D162" s="2">
@@ -2970,7 +2983,7 @@
       <c r="B163" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C163">
+      <c r="C163" s="3">
         <v>3112.4463999999998</v>
       </c>
       <c r="D163" s="2">
@@ -2984,7 +2997,7 @@
       <c r="B164" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C164">
+      <c r="C164" s="3">
         <v>619.04640000000006</v>
       </c>
       <c r="D164" s="2">
@@ -2998,7 +3011,7 @@
       <c r="B165" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C165">
+      <c r="C165" s="3">
         <v>1096.5136</v>
       </c>
       <c r="D165" s="2">
@@ -3012,7 +3025,7 @@
       <c r="B166" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C166">
+      <c r="C166" s="3">
         <v>1789.7152000000001</v>
       </c>
       <c r="D166" s="2">
@@ -3026,7 +3039,7 @@
       <c r="B167" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C167">
+      <c r="C167" s="3">
         <v>1600.3008</v>
       </c>
       <c r="D167" s="2">
@@ -3040,7 +3053,7 @@
       <c r="B168" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C168">
+      <c r="C168" s="3">
         <v>1573.9584</v>
       </c>
       <c r="D168" s="2">
@@ -3054,7 +3067,7 @@
       <c r="B169" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C169">
+      <c r="C169" s="3">
         <v>3838.4639999999999</v>
       </c>
       <c r="D169" s="2">
@@ -3068,7 +3081,7 @@
       <c r="B170" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C170">
+      <c r="C170" s="3">
         <v>2907.6656000000003</v>
       </c>
       <c r="D170" s="2">
@@ -3082,7 +3095,7 @@
       <c r="B171" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C171">
+      <c r="C171" s="3">
         <v>152.88</v>
       </c>
       <c r="D171" s="2">
@@ -3096,7 +3109,7 @@
       <c r="B172" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C172">
+      <c r="C172" s="3">
         <v>3153.8751999999999</v>
       </c>
       <c r="D172" s="2">
@@ -3110,7 +3123,7 @@
       <c r="B173" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C173">
+      <c r="C173" s="3">
         <v>5317.4016000000001</v>
       </c>
       <c r="D173" s="2">
@@ -3124,7 +3137,7 @@
       <c r="B174" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C174">
+      <c r="C174" s="3">
         <v>421.47839999999997</v>
       </c>
       <c r="D174" s="2">
@@ -3138,7 +3151,7 @@
       <c r="B175" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C175">
+      <c r="C175" s="3">
         <v>2736.1152000000002</v>
       </c>
       <c r="D175" s="2">
@@ -3152,7 +3165,7 @@
       <c r="B176" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C176">
+      <c r="C176" s="3">
         <v>882</v>
       </c>
       <c r="D176" s="2">
@@ -3166,7 +3179,7 @@
       <c r="B177" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C177">
+      <c r="C177" s="3">
         <v>5005.0560000000005</v>
       </c>
       <c r="D177" s="2">
@@ -3180,7 +3193,7 @@
       <c r="B178" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C178">
+      <c r="C178" s="3">
         <v>12189.374400000001</v>
       </c>
       <c r="D178" s="2">
@@ -3194,7 +3207,7 @@
       <c r="B179" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C179">
+      <c r="C179" s="3">
         <v>1072.2208000000001</v>
       </c>
       <c r="D179" s="2">
@@ -3208,7 +3221,7 @@
       <c r="B180" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C180">
+      <c r="C180" s="3">
         <v>12139.814400000001</v>
       </c>
       <c r="D180" s="2">
@@ -3222,7 +3235,7 @@
       <c r="B181" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C181">
+      <c r="C181" s="3">
         <v>225.792</v>
       </c>
       <c r="D181" s="2">
@@ -3236,7 +3249,7 @@
       <c r="B182" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C182">
+      <c r="C182" s="3">
         <v>926.45280000000002</v>
       </c>
       <c r="D182" s="2">
@@ -3250,7 +3263,7 @@
       <c r="B183" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C183">
+      <c r="C183" s="3">
         <v>997.39359999999999</v>
       </c>
       <c r="D183" s="2">
@@ -3264,7 +3277,7 @@
       <c r="B184" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C184">
+      <c r="C184" s="3">
         <v>465.69600000000003</v>
       </c>
       <c r="D184" s="2">
@@ -3278,7 +3291,7 @@
       <c r="B185" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C185">
+      <c r="C185" s="3">
         <v>750.75840000000005</v>
       </c>
       <c r="D185" s="2">
@@ -3292,7 +3305,7 @@
       <c r="B186" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C186">
+      <c r="C186" s="3">
         <v>1250.7583999999999</v>
       </c>
       <c r="D186" s="2">
@@ -3306,7 +3319,7 @@
       <c r="B187" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C187">
+      <c r="C187" s="3">
         <v>6988.9791999999998</v>
       </c>
       <c r="D187" s="2">
@@ -3320,7 +3333,7 @@
       <c r="B188" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C188">
+      <c r="C188" s="3">
         <v>4631.3231999999998</v>
       </c>
       <c r="D188" s="2">
@@ -3334,7 +3347,7 @@
       <c r="B189" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C189">
+      <c r="C189" s="3">
         <v>953.97119999999995</v>
       </c>
       <c r="D189" s="2">
@@ -3348,7 +3361,7 @@
       <c r="B190" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C190">
+      <c r="C190" s="3">
         <v>4332.4960000000001</v>
       </c>
       <c r="D190" s="2">
@@ -3362,7 +3375,7 @@
       <c r="B191" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C191">
+      <c r="C191" s="3">
         <v>17608.9984</v>
       </c>
       <c r="D191" s="2">
@@ -3376,7 +3389,7 @@
       <c r="B192" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C192">
+      <c r="C192" s="3">
         <v>1074.472</v>
       </c>
       <c r="D192" s="2">
@@ -3390,7 +3403,7 @@
       <c r="B193" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C193">
+      <c r="C193" s="3">
         <v>2074.4720000000002</v>
       </c>
       <c r="D193" s="2">
@@ -3404,7 +3417,7 @@
       <c r="B194" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C194">
+      <c r="C194" s="3">
         <v>430.08</v>
       </c>
       <c r="D194" s="2">
@@ -3418,7 +3431,7 @@
       <c r="B195" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C195">
+      <c r="C195" s="3">
         <v>12793.267199999998</v>
       </c>
       <c r="D195" s="2">
@@ -3432,7 +3445,7 @@
       <c r="B196" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C196">
+      <c r="C196" s="3">
         <v>3824.2736000000004</v>
       </c>
       <c r="D196" s="2">
@@ -3446,7 +3459,7 @@
       <c r="B197" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C197">
+      <c r="C197" s="3">
         <v>632.76639999999998</v>
       </c>
       <c r="D197" s="2">
@@ -3460,7 +3473,7 @@
       <c r="B198" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C198">
+      <c r="C198" s="3">
         <v>4499.9696000000004</v>
       </c>
       <c r="D198" s="2">
@@ -3474,7 +3487,7 @@
       <c r="B199" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C199">
+      <c r="C199" s="3">
         <v>2499.9695999999999</v>
       </c>
       <c r="D199" s="2">
@@ -3488,7 +3501,7 @@
       <c r="B200" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C200">
+      <c r="C200" s="3">
         <v>2712.0128</v>
       </c>
       <c r="D200" s="2">
@@ -3502,7 +3515,7 @@
       <c r="B201" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C201">
+      <c r="C201" s="3">
         <v>5362.5599999999995</v>
       </c>
       <c r="D201" s="2">
@@ -3516,7 +3529,7 @@
       <c r="B202" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C202">
+      <c r="C202" s="3">
         <v>490.84</v>
       </c>
       <c r="D202" s="2">
@@ -3530,7 +3543,7 @@
       <c r="B203" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C203">
+      <c r="C203" s="3">
         <v>3908.0832</v>
       </c>
       <c r="D203" s="2">
@@ -3544,7 +3557,7 @@
       <c r="B204" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C204">
+      <c r="C204" s="3">
         <v>2591.9039999999995</v>
       </c>
       <c r="D204" s="2">
@@ -3558,7 +3571,7 @@
       <c r="B205" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C205">
+      <c r="C205" s="3">
         <v>3189.6480000000001</v>
       </c>
       <c r="D205" s="2">
@@ -3572,7 +3585,7 @@
       <c r="B206" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C206">
+      <c r="C206" s="3">
         <v>70.56</v>
       </c>
       <c r="D206" s="2">
@@ -3586,7 +3599,7 @@
       <c r="B207" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C207">
+      <c r="C207" s="3">
         <v>2411.3712</v>
       </c>
       <c r="D207" s="2">

</xml_diff>